<commit_message>
Start returns at first period after idea date
</commit_message>
<xml_diff>
--- a/analysis/forward_beat_curves.xlsx
+++ b/analysis/forward_beat_curves.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="Rc1d2c6f5dc124dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="R52bdd28c3c6d4fc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85efa81628414f1c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R945f0d7a8d7449cc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -811,40 +811,40 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="C2" s="4" t="n">
-        <x:v>2.24823169</x:v>
+        <x:v>0.85347234</x:v>
       </x:c>
       <x:c r="D2" s="4" t="n">
-        <x:v>2.09684963</x:v>
+        <x:v>0.6964316100000001</x:v>
       </x:c>
       <x:c r="E2" s="4" t="n">
-        <x:v>0.25718404</x:v>
+        <x:v>0.2459711</x:v>
       </x:c>
       <x:c r="F2" s="4" t="n">
-        <x:v>0.11016848</x:v>
+        <x:v>0.0998978</x:v>
       </x:c>
       <x:c r="G2" s="4" t="n">
-        <x:v>13.251324810000002</x:v>
+        <x:v>1.2169218800000001</x:v>
       </x:c>
       <x:c r="H2" s="4" t="n">
-        <x:v>13.09311777</x:v>
+        <x:v>1.0729649399999999</x:v>
       </x:c>
       <x:c r="I2" s="4" t="n">
-        <x:v>0.36486362</x:v>
+        <x:v>0.41231779</x:v>
       </x:c>
       <x:c r="J2" s="4" t="n">
-        <x:v>0.22472991</x:v>
+        <x:v>0.33460306</x:v>
       </x:c>
       <x:c r="K2" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L2" s="5" t="n">
-        <x:v>3819</x:v>
+        <x:v>4311</x:v>
       </x:c>
       <x:c r="M2" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N2" s="5" t="n">
-        <x:v>193</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="O2" s="3" t="n">
         <x:v>0.25</x:v>
@@ -867,52 +867,52 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="C3" s="4" t="n">
-        <x:v>0.38118220999999997</x:v>
+        <x:v>0.49339219999999995</x:v>
       </x:c>
       <x:c r="D3" s="4" t="n">
-        <x:v>0.24759328</x:v>
+        <x:v>0.36687009000000004</x:v>
       </x:c>
       <x:c r="E3" s="4" t="n">
-        <x:v>0.0500009</x:v>
+        <x:v>0.04826066</x:v>
       </x:c>
       <x:c r="F3" s="4" t="n">
-        <x:v>-0.07124741</x:v>
+        <x:v>-0.07502689</x:v>
       </x:c>
       <x:c r="G3" s="4" t="n">
-        <x:v>1.5720725</x:v>
+        <x:v>0.47907014</x:v>
       </x:c>
       <x:c r="H3" s="4" t="n">
-        <x:v>1.44225412</x:v>
+        <x:v>0.36860315</x:v>
       </x:c>
       <x:c r="I3" s="4" t="n">
-        <x:v>0.11494623000000001</x:v>
+        <x:v>0.12950418</x:v>
       </x:c>
       <x:c r="J3" s="4" t="n">
-        <x:v>0.02211067</x:v>
+        <x:v>0.05005334</x:v>
       </x:c>
       <x:c r="K3" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L3" s="5" t="n">
-        <x:v>3747</x:v>
+        <x:v>4225</x:v>
       </x:c>
       <x:c r="M3" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N3" s="5" t="n">
-        <x:v>185</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="O3" s="3" t="n">
-        <x:v>0.496019</x:v>
+        <x:v>0.496431</x:v>
       </x:c>
       <x:c r="P3" s="3" t="n">
-        <x:v>0.498732</x:v>
+        <x:v>0.497574</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="n">
-        <x:v>0.490132</x:v>
+        <x:v>0.494624</x:v>
       </x:c>
       <x:c r="R3" s="3" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.496849</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -923,52 +923,52 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
-        <x:v>0.23069671</x:v>
+        <x:v>0.22641802</x:v>
       </x:c>
       <x:c r="D4" s="4" t="n">
-        <x:v>0.10602118</x:v>
+        <x:v>0.10375677</x:v>
       </x:c>
       <x:c r="E4" s="4" t="n">
-        <x:v>-0.00978715</x:v>
+        <x:v>-0.00716369</x:v>
       </x:c>
       <x:c r="F4" s="4" t="n">
-        <x:v>-0.12657378</x:v>
+        <x:v>-0.12250541999999999</x:v>
       </x:c>
       <x:c r="G4" s="4" t="n">
-        <x:v>0.89143337</x:v>
+        <x:v>0.36874591</x:v>
       </x:c>
       <x:c r="H4" s="4" t="n">
-        <x:v>0.7858886599999999</x:v>
+        <x:v>0.27277081</x:v>
       </x:c>
       <x:c r="I4" s="4" t="n">
-        <x:v>0.06245528</x:v>
+        <x:v>0.05197191</x:v>
       </x:c>
       <x:c r="J4" s="4" t="n">
-        <x:v>-0.03363994</x:v>
+        <x:v>-0.03351134</x:v>
       </x:c>
       <x:c r="K4" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L4" s="5" t="n">
-        <x:v>3659</x:v>
+        <x:v>4133</x:v>
       </x:c>
       <x:c r="M4" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N4" s="5" t="n">
-        <x:v>171</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="O4" s="3" t="n">
-        <x:v>0.739352</x:v>
+        <x:v>0.73921</x:v>
       </x:c>
       <x:c r="P4" s="3" t="n">
-        <x:v>0.745217</x:v>
+        <x:v>0.743104</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="n">
-        <x:v>0.726974</x:v>
+        <x:v>0.739247</x:v>
       </x:c>
       <x:c r="R4" s="3" t="n">
-        <x:v>0.747076</x:v>
+        <x:v>0.742257</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -979,52 +979,52 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
-        <x:v>0.1529898</x:v>
+        <x:v>0.13736392</x:v>
       </x:c>
       <x:c r="D5" s="4" t="n">
-        <x:v>0.03237439</x:v>
+        <x:v>0.01986067</x:v>
       </x:c>
       <x:c r="E5" s="4" t="n">
-        <x:v>-0.02741681</x:v>
+        <x:v>-0.02318709</x:v>
       </x:c>
       <x:c r="F5" s="4" t="n">
-        <x:v>-0.13809864</x:v>
+        <x:v>-0.13263824</x:v>
       </x:c>
       <x:c r="G5" s="4" t="n">
-        <x:v>0.62289695</x:v>
+        <x:v>0.25046365000000004</x:v>
       </x:c>
       <x:c r="H5" s="4" t="n">
-        <x:v>0.5293873099999999</x:v>
+        <x:v>0.17084428</x:v>
       </x:c>
       <x:c r="I5" s="4" t="n">
-        <x:v>0.019454469999999998</x:v>
+        <x:v>0.03826666</x:v>
       </x:c>
       <x:c r="J5" s="4" t="n">
-        <x:v>-0.06953677</x:v>
+        <x:v>-0.04164593</x:v>
       </x:c>
       <x:c r="K5" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L5" s="5" t="n">
-        <x:v>3563</x:v>
+        <x:v>4032</x:v>
       </x:c>
       <x:c r="M5" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N5" s="5" t="n">
-        <x:v>168</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="O5" s="3" t="n">
-        <x:v>0.979537</x:v>
+        <x:v>0.978586</x:v>
       </x:c>
       <x:c r="P5" s="3" t="n">
-        <x:v>0.990247</x:v>
+        <x:v>0.986235</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="n">
-        <x:v>0.963816</x:v>
+        <x:v>0.975806</x:v>
       </x:c>
       <x:c r="R5" s="3" t="n">
-        <x:v>0.99256</x:v>
+        <x:v>0.984163</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1035,52 +1035,52 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
-        <x:v>0.11798879</x:v>
+        <x:v>0.10771236000000001</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
-        <x:v>0.00002065</x:v>
+        <x:v>-0.01146338</x:v>
       </x:c>
       <x:c r="E6" s="4" t="n">
-        <x:v>-0.04103339</x:v>
+        <x:v>-0.042991549999999996</x:v>
       </x:c>
       <x:c r="F6" s="4" t="n">
-        <x:v>-0.15179735</x:v>
+        <x:v>-0.1521901</x:v>
       </x:c>
       <x:c r="G6" s="4" t="n">
-        <x:v>0.52018017</x:v>
+        <x:v>0.19265449</x:v>
       </x:c>
       <x:c r="H6" s="4" t="n">
-        <x:v>0.43496505999999996</x:v>
+        <x:v>0.11189301</x:v>
       </x:c>
       <x:c r="I6" s="4" t="n">
-        <x:v>0.0081421</x:v>
+        <x:v>-0.00557066</x:v>
       </x:c>
       <x:c r="J6" s="4" t="n">
-        <x:v>-0.08539844</x:v>
+        <x:v>-0.09169290000000001</x:v>
       </x:c>
       <x:c r="K6" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L6" s="5" t="n">
-        <x:v>3515</x:v>
+        <x:v>3995</x:v>
       </x:c>
       <x:c r="M6" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N6" s="5" t="n">
-        <x:v>166</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="O6" s="3" t="n">
-        <x:v>1.216111</x:v>
+        <x:v>1.213811</x:v>
       </x:c>
       <x:c r="P6" s="3" t="n">
-        <x:v>1.233642</x:v>
+        <x:v>1.22622</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="n">
-        <x:v>1.1875</x:v>
+        <x:v>1.204301</x:v>
       </x:c>
       <x:c r="R6" s="3" t="n">
-        <x:v>1.237952</x:v>
+        <x:v>1.221973</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1091,52 +1091,52 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
-        <x:v>0.09919385</x:v>
+        <x:v>0.08246974</x:v>
       </x:c>
       <x:c r="D7" s="4" t="n">
-        <x:v>-0.019649859999999998</x:v>
+        <x:v>-0.03681151</x:v>
       </x:c>
       <x:c r="E7" s="4" t="n">
-        <x:v>-0.04563599</x:v>
+        <x:v>-0.04169284</x:v>
       </x:c>
       <x:c r="F7" s="4" t="n">
-        <x:v>-0.15583248</x:v>
+        <x:v>-0.15062669</x:v>
       </x:c>
       <x:c r="G7" s="4" t="n">
-        <x:v>0.43358129</x:v>
+        <x:v>0.17351121</x:v>
       </x:c>
       <x:c r="H7" s="4" t="n">
-        <x:v>0.3421975</x:v>
+        <x:v>0.08579101</x:v>
       </x:c>
       <x:c r="I7" s="4" t="n">
-        <x:v>0.00952176</x:v>
+        <x:v>-0.00854878</x:v>
       </x:c>
       <x:c r="J7" s="4" t="n">
-        <x:v>-0.07935047</x:v>
+        <x:v>-0.09121974</x:v>
       </x:c>
       <x:c r="K7" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L7" s="5" t="n">
-        <x:v>3446</x:v>
+        <x:v>3880</x:v>
       </x:c>
       <x:c r="M7" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N7" s="5" t="n">
-        <x:v>162</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="O7" s="3" t="n">
-        <x:v>1.449074</x:v>
+        <x:v>1.445634</x:v>
       </x:c>
       <x:c r="P7" s="3" t="n">
-        <x:v>1.474028</x:v>
+        <x:v>1.463338</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="n">
-        <x:v>1.404605</x:v>
+        <x:v>1.427419</x:v>
       </x:c>
       <x:c r="R7" s="3" t="n">
-        <x:v>1.479938</x:v>
+        <x:v>1.455069</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1147,52 +1147,52 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
-        <x:v>0.08291791</x:v>
+        <x:v>0.06626699999999999</x:v>
       </x:c>
       <x:c r="D8" s="4" t="n">
-        <x:v>-0.03743142</x:v>
+        <x:v>-0.054786339999999996</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
-        <x:v>-0.046157250000000004</x:v>
+        <x:v>-0.04097415</x:v>
       </x:c>
       <x:c r="F8" s="4" t="n">
-        <x:v>-0.15784511</x:v>
+        <x:v>-0.15183603</x:v>
       </x:c>
       <x:c r="G8" s="4" t="n">
-        <x:v>0.38998500999999997</x:v>
+        <x:v>0.17618944</x:v>
       </x:c>
       <x:c r="H8" s="4" t="n">
-        <x:v>0.30150953999999996</x:v>
+        <x:v>0.08293892</x:v>
       </x:c>
       <x:c r="I8" s="4" t="n">
-        <x:v>-0.00872581</x:v>
+        <x:v>-0.01890776</x:v>
       </x:c>
       <x:c r="J8" s="4" t="n">
-        <x:v>-0.10121532999999999</x:v>
+        <x:v>-0.10660539999999999</x:v>
       </x:c>
       <x:c r="K8" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L8" s="5" t="n">
-        <x:v>3387</x:v>
+        <x:v>3827</x:v>
       </x:c>
       <x:c r="M8" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N8" s="5" t="n">
-        <x:v>161</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="O8" s="3" t="n">
-        <x:v>1.679537</x:v>
+        <x:v>1.67422</x:v>
       </x:c>
       <x:c r="P8" s="3" t="n">
-        <x:v>1.712135</x:v>
+        <x:v>1.698132</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="n">
-        <x:v>1.621711</x:v>
+        <x:v>1.647849</x:v>
       </x:c>
       <x:c r="R8" s="3" t="n">
-        <x:v>1.720497</x:v>
+        <x:v>1.688657</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1203,52 +1203,52 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="4" t="n">
-        <x:v>0.07342061</x:v>
+        <x:v>0.05637983</x:v>
       </x:c>
       <x:c r="D9" s="4" t="n">
-        <x:v>-0.047021610000000005</x:v>
+        <x:v>-0.06464265</x:v>
       </x:c>
       <x:c r="E9" s="4" t="n">
-        <x:v>-0.04452318</x:v>
+        <x:v>-0.040083799999999996</x:v>
       </x:c>
       <x:c r="F9" s="4" t="n">
-        <x:v>-0.15668238</x:v>
+        <x:v>-0.14934551000000001</x:v>
       </x:c>
       <x:c r="G9" s="4" t="n">
-        <x:v>0.38189366</x:v>
+        <x:v>0.17343931</x:v>
       </x:c>
       <x:c r="H9" s="4" t="n">
-        <x:v>0.2870739</x:v>
+        <x:v>0.07613233</x:v>
       </x:c>
       <x:c r="I9" s="4" t="n">
-        <x:v>0.00083387</x:v>
+        <x:v>-0.009557949999999999</x:v>
       </x:c>
       <x:c r="J9" s="4" t="n">
-        <x:v>-0.0897294</x:v>
+        <x:v>-0.09540971000000001</x:v>
       </x:c>
       <x:c r="K9" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L9" s="5" t="n">
-        <x:v>3341</x:v>
+        <x:v>3761</x:v>
       </x:c>
       <x:c r="M9" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N9" s="5" t="n">
-        <x:v>161</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="O9" s="3" t="n">
-        <x:v>1.907222</x:v>
+        <x:v>1.899485</x:v>
       </x:c>
       <x:c r="P9" s="3" t="n">
-        <x:v>1.948294</x:v>
+        <x:v>1.92954</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="n">
-        <x:v>1.838816</x:v>
+        <x:v>1.862903</x:v>
       </x:c>
       <x:c r="R9" s="3" t="n">
-        <x:v>1.96118</x:v>
+        <x:v>1.916274</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1259,52 +1259,52 @@
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="C10" s="4" t="n">
-        <x:v>0.06485229</x:v>
+        <x:v>0.05137715</x:v>
       </x:c>
       <x:c r="D10" s="4" t="n">
-        <x:v>-0.05614853</x:v>
+        <x:v>-0.07025210999999999</x:v>
       </x:c>
       <x:c r="E10" s="4" t="n">
-        <x:v>-0.04856356</x:v>
+        <x:v>-0.04344598</x:v>
       </x:c>
       <x:c r="F10" s="4" t="n">
-        <x:v>-0.16062328999999997</x:v>
+        <x:v>-0.15553213</x:v>
       </x:c>
       <x:c r="G10" s="4" t="n">
-        <x:v>0.3408206</x:v>
+        <x:v>0.17047443</x:v>
       </x:c>
       <x:c r="H10" s="4" t="n">
-        <x:v>0.24808847</x:v>
+        <x:v>0.07508491</x:v>
       </x:c>
       <x:c r="I10" s="4" t="n">
-        <x:v>0.00028314</x:v>
+        <x:v>-0.01441129</x:v>
       </x:c>
       <x:c r="J10" s="4" t="n">
-        <x:v>-0.08441209000000001</x:v>
+        <x:v>-0.09647681000000001</x:v>
       </x:c>
       <x:c r="K10" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L10" s="5" t="n">
-        <x:v>3309</x:v>
+        <x:v>3710</x:v>
       </x:c>
       <x:c r="M10" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N10" s="5" t="n">
-        <x:v>159</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="O10" s="3" t="n">
-        <x:v>2.131481</x:v>
+        <x:v>2.121182</x:v>
       </x:c>
       <x:c r="P10" s="3" t="n">
-        <x:v>2.181701</x:v>
+        <x:v>2.15748</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="n">
-        <x:v>2.046053</x:v>
+        <x:v>2.072581</x:v>
       </x:c>
       <x:c r="R10" s="3" t="n">
-        <x:v>2.199686</x:v>
+        <x:v>2.139423</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1315,52 +1315,52 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="C11" s="4" t="n">
-        <x:v>0.05903213</x:v>
+        <x:v>0.04965592</x:v>
       </x:c>
       <x:c r="D11" s="4" t="n">
-        <x:v>-0.06250963999999999</x:v>
+        <x:v>-0.07374802</x:v>
       </x:c>
       <x:c r="E11" s="4" t="n">
-        <x:v>-0.04618363</x:v>
+        <x:v>-0.04364621</x:v>
       </x:c>
       <x:c r="F11" s="4" t="n">
-        <x:v>-0.15901998</x:v>
+        <x:v>-0.15694091</x:v>
       </x:c>
       <x:c r="G11" s="4" t="n">
-        <x:v>0.33828068</x:v>
+        <x:v>0.17915729</x:v>
       </x:c>
       <x:c r="H11" s="4" t="n">
-        <x:v>0.24771844999999998</x:v>
+        <x:v>0.08557295999999999</x:v>
       </x:c>
       <x:c r="I11" s="4" t="n">
-        <x:v>0.00320646</x:v>
+        <x:v>0.00129888</x:v>
       </x:c>
       <x:c r="J11" s="4" t="n">
-        <x:v>-0.08032844</x:v>
+        <x:v>-0.08099233</x:v>
       </x:c>
       <x:c r="K11" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L11" s="5" t="n">
-        <x:v>3246</x:v>
+        <x:v>3674</x:v>
       </x:c>
       <x:c r="M11" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N11" s="5" t="n">
-        <x:v>156</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="O11" s="3" t="n">
-        <x:v>2.352685</x:v>
+        <x:v>2.338977</x:v>
       </x:c>
       <x:c r="P11" s="3" t="n">
-        <x:v>2.411121</x:v>
+        <x:v>2.381328</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="n">
-        <x:v>2.246711</x:v>
+        <x:v>2.276882</x:v>
       </x:c>
       <x:c r="R11" s="3" t="n">
-        <x:v>2.434295</x:v>
+        <x:v>2.356436</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1371,52 +1371,52 @@
         <x:v>2.75</x:v>
       </x:c>
       <x:c r="C12" s="4" t="n">
-        <x:v>0.060910469999999994</x:v>
+        <x:v>0.047061080000000005</x:v>
       </x:c>
       <x:c r="D12" s="4" t="n">
-        <x:v>-0.06244242</x:v>
+        <x:v>-0.07775604</x:v>
       </x:c>
       <x:c r="E12" s="4" t="n">
-        <x:v>-0.042021670000000004</x:v>
+        <x:v>-0.038533979999999995</x:v>
       </x:c>
       <x:c r="F12" s="4" t="n">
-        <x:v>-0.15588558</x:v>
+        <x:v>-0.15319107</x:v>
       </x:c>
       <x:c r="G12" s="4" t="n">
-        <x:v>0.32654451</x:v>
+        <x:v>0.16950151000000002</x:v>
       </x:c>
       <x:c r="H12" s="4" t="n">
-        <x:v>0.23519313</x:v>
+        <x:v>0.07227424</x:v>
       </x:c>
       <x:c r="I12" s="4" t="n">
-        <x:v>0.01126969</x:v>
+        <x:v>-0.0027602900000000003</x:v>
       </x:c>
       <x:c r="J12" s="4" t="n">
-        <x:v>-0.06969739</x:v>
+        <x:v>-0.08650550000000001</x:v>
       </x:c>
       <x:c r="K12" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L12" s="5" t="n">
-        <x:v>3210</x:v>
+        <x:v>3605</x:v>
       </x:c>
       <x:c r="M12" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N12" s="5" t="n">
-        <x:v>149</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="O12" s="3" t="n">
-        <x:v>2.570556</x:v>
+        <x:v>2.553038</x:v>
       </x:c>
       <x:c r="P12" s="3" t="n">
-        <x:v>2.638084</x:v>
+        <x:v>2.60104</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="n">
-        <x:v>2.447368</x:v>
+        <x:v>2.481183</x:v>
       </x:c>
       <x:c r="R12" s="3" t="n">
-        <x:v>2.66443</x:v>
+        <x:v>2.569797</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1427,52 +1427,52 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="4" t="n">
-        <x:v>0.05796689</x:v>
+        <x:v>0.04521357</x:v>
       </x:c>
       <x:c r="D13" s="4" t="n">
-        <x:v>-0.06673396000000001</x:v>
+        <x:v>-0.08095808</x:v>
       </x:c>
       <x:c r="E13" s="4" t="n">
-        <x:v>-0.04366314</x:v>
+        <x:v>-0.03737669</x:v>
       </x:c>
       <x:c r="F13" s="4" t="n">
-        <x:v>-0.15814809</x:v>
+        <x:v>-0.15223486</x:v>
       </x:c>
       <x:c r="G13" s="4" t="n">
-        <x:v>0.30185975</x:v>
+        <x:v>0.15899267</x:v>
       </x:c>
       <x:c r="H13" s="4" t="n">
-        <x:v>0.21080369000000002</x:v>
+        <x:v>0.06270749</x:v>
       </x:c>
       <x:c r="I13" s="4" t="n">
-        <x:v>0.02379598</x:v>
+        <x:v>0.004547590000000001</x:v>
       </x:c>
       <x:c r="J13" s="4" t="n">
-        <x:v>-0.05835143</x:v>
+        <x:v>-0.07835721999999999</x:v>
       </x:c>
       <x:c r="K13" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L13" s="5" t="n">
-        <x:v>3186</x:v>
+        <x:v>3565</x:v>
       </x:c>
       <x:c r="M13" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N13" s="5" t="n">
-        <x:v>147</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="O13" s="3" t="n">
-        <x:v>2.784907</x:v>
+        <x:v>2.761454</x:v>
       </x:c>
       <x:c r="P13" s="3" t="n">
-        <x:v>2.86268</x:v>
+        <x:v>2.81669</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="n">
-        <x:v>2.648026</x:v>
+        <x:v>2.682796</x:v>
       </x:c>
       <x:c r="R13" s="3" t="n">
-        <x:v>2.892857</x:v>
+        <x:v>2.78125</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1483,52 +1483,52 @@
         <x:v>3.25</x:v>
       </x:c>
       <x:c r="C14" s="4" t="n">
-        <x:v>0.05444923</x:v>
+        <x:v>0.04292559</x:v>
       </x:c>
       <x:c r="D14" s="4" t="n">
-        <x:v>-0.07138751</x:v>
+        <x:v>-0.08344895</x:v>
       </x:c>
       <x:c r="E14" s="4" t="n">
-        <x:v>-0.0394565</x:v>
+        <x:v>-0.03522115</x:v>
       </x:c>
       <x:c r="F14" s="4" t="n">
-        <x:v>-0.15493949</x:v>
+        <x:v>-0.15182003</x:v>
       </x:c>
       <x:c r="G14" s="4" t="n">
-        <x:v>0.29506779</x:v>
+        <x:v>0.14707031</x:v>
       </x:c>
       <x:c r="H14" s="4" t="n">
-        <x:v>0.20091024999999998</x:v>
+        <x:v>0.05222408</x:v>
       </x:c>
       <x:c r="I14" s="4" t="n">
-        <x:v>0.0157357</x:v>
+        <x:v>0.00970851</x:v>
       </x:c>
       <x:c r="J14" s="4" t="n">
-        <x:v>-0.06947901</x:v>
+        <x:v>-0.07890535</x:v>
       </x:c>
       <x:c r="K14" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L14" s="5" t="n">
-        <x:v>3115</x:v>
+        <x:v>3501</x:v>
       </x:c>
       <x:c r="M14" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N14" s="5" t="n">
-        <x:v>144</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="O14" s="3" t="n">
-        <x:v>2.99287</x:v>
+        <x:v>2.961404</x:v>
       </x:c>
       <x:c r="P14" s="3" t="n">
-        <x:v>3.078892</x:v>
+        <x:v>3.02435</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="n">
-        <x:v>2.845395</x:v>
+        <x:v>2.884409</x:v>
       </x:c>
       <x:c r="R14" s="3" t="n">
-        <x:v>3.118056</x:v>
+        <x:v>2.990741</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1539,52 +1539,52 @@
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="C15" s="4" t="n">
-        <x:v>0.052884650000000005</x:v>
+        <x:v>0.042789419999999995</x:v>
       </x:c>
       <x:c r="D15" s="4" t="n">
-        <x:v>-0.07296469</x:v>
+        <x:v>-0.08392604000000001</x:v>
       </x:c>
       <x:c r="E15" s="4" t="n">
-        <x:v>-0.03786627</x:v>
+        <x:v>-0.035603340000000004</x:v>
       </x:c>
       <x:c r="F15" s="4" t="n">
-        <x:v>-0.15410417</x:v>
+        <x:v>-0.15328917</x:v>
       </x:c>
       <x:c r="G15" s="4" t="n">
-        <x:v>0.27885508000000003</x:v>
+        <x:v>0.13447578999999998</x:v>
       </x:c>
       <x:c r="H15" s="4" t="n">
-        <x:v>0.18524174999999998</x:v>
+        <x:v>0.04044038</x:v>
       </x:c>
       <x:c r="I15" s="4" t="n">
-        <x:v>0.013165020000000001</x:v>
+        <x:v>-0.00387749</x:v>
       </x:c>
       <x:c r="J15" s="4" t="n">
-        <x:v>-0.07203282</x:v>
+        <x:v>-0.09157897999999999</x:v>
       </x:c>
       <x:c r="K15" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L15" s="5" t="n">
-        <x:v>3061</x:v>
+        <x:v>3467</x:v>
       </x:c>
       <x:c r="M15" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N15" s="5" t="n">
-        <x:v>144</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="O15" s="3" t="n">
-        <x:v>3.190926</x:v>
+        <x:v>3.154382</x:v>
       </x:c>
       <x:c r="P15" s="3" t="n">
-        <x:v>3.288549</x:v>
+        <x:v>3.227502</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="n">
-        <x:v>3.042763</x:v>
+        <x:v>3.086022</x:v>
       </x:c>
       <x:c r="R15" s="3" t="n">
-        <x:v>3.345486</x:v>
+        <x:v>3.195767</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1595,52 +1595,52 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="C16" s="4" t="n">
-        <x:v>0.05167694</x:v>
+        <x:v>0.03997842</x:v>
       </x:c>
       <x:c r="D16" s="4" t="n">
-        <x:v>-0.07487475</x:v>
+        <x:v>-0.08785631</x:v>
       </x:c>
       <x:c r="E16" s="4" t="n">
-        <x:v>-0.038357869999999995</x:v>
+        <x:v>-0.03434762</x:v>
       </x:c>
       <x:c r="F16" s="4" t="n">
-        <x:v>-0.15546027</x:v>
+        <x:v>-0.15284767</x:v>
       </x:c>
       <x:c r="G16" s="4" t="n">
-        <x:v>0.25538304</x:v>
+        <x:v>0.12694901</x:v>
       </x:c>
       <x:c r="H16" s="4" t="n">
-        <x:v>0.16269943</x:v>
+        <x:v>0.02907465</x:v>
       </x:c>
       <x:c r="I16" s="4" t="n">
-        <x:v>-0.01744938</x:v>
+        <x:v>-0.019802709999999998</x:v>
       </x:c>
       <x:c r="J16" s="4" t="n">
-        <x:v>-0.10291204000000001</x:v>
+        <x:v>-0.10766265000000001</x:v>
       </x:c>
       <x:c r="K16" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L16" s="5" t="n">
-        <x:v>3045</x:v>
+        <x:v>3435</x:v>
       </x:c>
       <x:c r="M16" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N16" s="5" t="n">
-        <x:v>145</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="O16" s="3" t="n">
-        <x:v>3.382407</x:v>
+        <x:v>3.339309</x:v>
       </x:c>
       <x:c r="P16" s="3" t="n">
-        <x:v>3.49335</x:v>
+        <x:v>3.423217</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="n">
-        <x:v>3.240132</x:v>
+        <x:v>3.284946</x:v>
       </x:c>
       <x:c r="R16" s="3" t="n">
-        <x:v>3.565517</x:v>
+        <x:v>3.396277</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1651,52 +1651,52 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C17" s="4" t="n">
-        <x:v>0.04870494</x:v>
+        <x:v>0.03864675</x:v>
       </x:c>
       <x:c r="D17" s="4" t="n">
-        <x:v>-0.07866987</x:v>
+        <x:v>-0.0894955</x:v>
       </x:c>
       <x:c r="E17" s="4" t="n">
-        <x:v>-0.03246901</x:v>
+        <x:v>-0.030030739999999997</x:v>
       </x:c>
       <x:c r="F17" s="4" t="n">
-        <x:v>-0.15016864</x:v>
+        <x:v>-0.14920912</x:v>
       </x:c>
       <x:c r="G17" s="4" t="n">
-        <x:v>0.24601140000000002</x:v>
+        <x:v>0.11463459999999999</x:v>
       </x:c>
       <x:c r="H17" s="4" t="n">
-        <x:v>0.14919665000000001</x:v>
+        <x:v>0.0168668</x:v>
       </x:c>
       <x:c r="I17" s="4" t="n">
-        <x:v>0.0019126000000000002</x:v>
+        <x:v>-0.007529559999999999</x:v>
       </x:c>
       <x:c r="J17" s="4" t="n">
-        <x:v>-0.08682121999999999</x:v>
+        <x:v>-0.10031411</x:v>
       </x:c>
       <x:c r="K17" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L17" s="5" t="n">
-        <x:v>2986</x:v>
+        <x:v>3370</x:v>
       </x:c>
       <x:c r="M17" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N17" s="5" t="n">
-        <x:v>138</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="O17" s="3" t="n">
-        <x:v>3.565463</x:v>
+        <x:v>3.516766</x:v>
       </x:c>
       <x:c r="P17" s="3" t="n">
-        <x:v>3.686956</x:v>
+        <x:v>3.607864</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="n">
-        <x:v>3.434211</x:v>
+        <x:v>3.475806</x:v>
       </x:c>
       <x:c r="R17" s="3" t="n">
-        <x:v>3.771739</x:v>
+        <x:v>3.579167</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1707,52 +1707,52 @@
         <x:v>4.25</x:v>
       </x:c>
       <x:c r="C18" s="4" t="n">
-        <x:v>0.04797001</x:v>
+        <x:v>0.03851088</x:v>
       </x:c>
       <x:c r="D18" s="4" t="n">
-        <x:v>-0.0795706</x:v>
+        <x:v>-0.09003164999999999</x:v>
       </x:c>
       <x:c r="E18" s="4" t="n">
-        <x:v>-0.03297468</x:v>
+        <x:v>-0.0324718</x:v>
       </x:c>
       <x:c r="F18" s="4" t="n">
-        <x:v>-0.15145261</x:v>
+        <x:v>-0.15249068</x:v>
       </x:c>
       <x:c r="G18" s="4" t="n">
-        <x:v>0.21806525000000002</x:v>
+        <x:v>0.10930662</x:v>
       </x:c>
       <x:c r="H18" s="4" t="n">
-        <x:v>0.12224317</x:v>
+        <x:v>0.009730879999999999</x:v>
       </x:c>
       <x:c r="I18" s="4" t="n">
-        <x:v>-0.0168384</x:v>
+        <x:v>-0.035756800000000005</x:v>
       </x:c>
       <x:c r="J18" s="4" t="n">
-        <x:v>-0.11122488000000001</x:v>
+        <x:v>-0.13275074</x:v>
       </x:c>
       <x:c r="K18" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L18" s="5" t="n">
-        <x:v>2954</x:v>
+        <x:v>3347</x:v>
       </x:c>
       <x:c r="M18" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N18" s="5" t="n">
-        <x:v>140</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="O18" s="3" t="n">
-        <x:v>3.741574</x:v>
+        <x:v>3.686421</x:v>
       </x:c>
       <x:c r="P18" s="3" t="n">
-        <x:v>3.875423</x:v>
+        <x:v>3.788766</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="n">
-        <x:v>3.621711</x:v>
+        <x:v>3.66129</x:v>
       </x:c>
       <x:c r="R18" s="3" t="n">
-        <x:v>3.9875</x:v>
+        <x:v>3.784946</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1763,52 +1763,52 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="C19" s="4" t="n">
-        <x:v>0.04677849</x:v>
+        <x:v>0.0379149</x:v>
       </x:c>
       <x:c r="D19" s="4" t="n">
-        <x:v>-0.08127632</x:v>
+        <x:v>-0.09101485000000001</x:v>
       </x:c>
       <x:c r="E19" s="4" t="n">
-        <x:v>-0.0317633</x:v>
+        <x:v>-0.02897285</x:v>
       </x:c>
       <x:c r="F19" s="4" t="n">
-        <x:v>-0.15081706</x:v>
+        <x:v>-0.14904006</x:v>
       </x:c>
       <x:c r="G19" s="4" t="n">
-        <x:v>0.20629269</x:v>
+        <x:v>0.10266954</x:v>
       </x:c>
       <x:c r="H19" s="4" t="n">
-        <x:v>0.1099639</x:v>
+        <x:v>0.0006900599999999999</x:v>
       </x:c>
       <x:c r="I19" s="4" t="n">
-        <x:v>-0.01721581</x:v>
+        <x:v>-0.01626404</x:v>
       </x:c>
       <x:c r="J19" s="4" t="n">
-        <x:v>-0.1137833</x:v>
+        <x:v>-0.11220707</x:v>
       </x:c>
       <x:c r="K19" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L19" s="5" t="n">
-        <x:v>2918</x:v>
+        <x:v>3301</x:v>
       </x:c>
       <x:c r="M19" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N19" s="5" t="n">
-        <x:v>138</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="O19" s="3" t="n">
-        <x:v>3.91037</x:v>
+        <x:v>3.849602</x:v>
       </x:c>
       <x:c r="P19" s="3" t="n">
-        <x:v>4.05646</x:v>
+        <x:v>3.958725</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="n">
-        <x:v>3.805921</x:v>
+        <x:v>3.841398</x:v>
       </x:c>
       <x:c r="R19" s="3" t="n">
-        <x:v>4.186594</x:v>
+        <x:v>3.952778</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1819,52 +1819,52 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="C20" s="4" t="n">
-        <x:v>0.046780249999999995</x:v>
+        <x:v>0.03778899</x:v>
       </x:c>
       <x:c r="D20" s="4" t="n">
-        <x:v>-0.08175044</x:v>
+        <x:v>-0.09095501</x:v>
       </x:c>
       <x:c r="E20" s="4" t="n">
-        <x:v>-0.02810962</x:v>
+        <x:v>-0.0258489</x:v>
       </x:c>
       <x:c r="F20" s="4" t="n">
-        <x:v>-0.14733241</x:v>
+        <x:v>-0.14638155</x:v>
       </x:c>
       <x:c r="G20" s="4" t="n">
-        <x:v>0.21110872</x:v>
+        <x:v>0.10434302000000001</x:v>
       </x:c>
       <x:c r="H20" s="4" t="n">
-        <x:v>0.11277879</x:v>
+        <x:v>0.0014299500000000001</x:v>
       </x:c>
       <x:c r="I20" s="4" t="n">
-        <x:v>-0.0034173999999999997</x:v>
+        <x:v>-0.01786274</x:v>
       </x:c>
       <x:c r="J20" s="4" t="n">
-        <x:v>-0.09378943</x:v>
+        <x:v>-0.11255651</x:v>
       </x:c>
       <x:c r="K20" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L20" s="5" t="n">
-        <x:v>2880</x:v>
+        <x:v>3259</x:v>
       </x:c>
       <x:c r="M20" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N20" s="5" t="n">
-        <x:v>135</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="O20" s="3" t="n">
-        <x:v>4.072593</x:v>
+        <x:v>4.005644</x:v>
       </x:c>
       <x:c r="P20" s="3" t="n">
-        <x:v>4.229427</x:v>
+        <x:v>4.12174</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="n">
-        <x:v>3.986842</x:v>
+        <x:v>4.010753</x:v>
       </x:c>
       <x:c r="R20" s="3" t="n">
-        <x:v>4.374074</x:v>
+        <x:v>4.125</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1875,52 +1875,52 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="4" t="n">
-        <x:v>0.046392569999999994</x:v>
+        <x:v>0.03901952</x:v>
       </x:c>
       <x:c r="D21" s="4" t="n">
-        <x:v>-0.08194342</x:v>
+        <x:v>-0.09000679</x:v>
       </x:c>
       <x:c r="E21" s="4" t="n">
-        <x:v>-0.02569775</x:v>
+        <x:v>-0.02469486</x:v>
       </x:c>
       <x:c r="F21" s="4" t="n">
-        <x:v>-0.1447298</x:v>
+        <x:v>-0.14580602</x:v>
       </x:c>
       <x:c r="G21" s="4" t="n">
-        <x:v>0.20167922000000002</x:v>
+        <x:v>0.10637718</x:v>
       </x:c>
       <x:c r="H21" s="4" t="n">
-        <x:v>0.10344272</x:v>
+        <x:v>0.00281159</x:v>
       </x:c>
       <x:c r="I21" s="4" t="n">
-        <x:v>-0.0130787</x:v>
+        <x:v>-0.01214491</x:v>
       </x:c>
       <x:c r="J21" s="4" t="n">
-        <x:v>-0.10493866</x:v>
+        <x:v>-0.10976285000000001</x:v>
       </x:c>
       <x:c r="K21" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L21" s="5" t="n">
-        <x:v>2850</x:v>
+        <x:v>3229</x:v>
       </x:c>
       <x:c r="M21" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N21" s="5" t="n">
-        <x:v>139</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="O21" s="3" t="n">
-        <x:v>4.228704</x:v>
+        <x:v>4.157122</x:v>
       </x:c>
       <x:c r="P21" s="3" t="n">
-        <x:v>4.397544</x:v>
+        <x:v>4.280118</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="n">
-        <x:v>4.161184</x:v>
+        <x:v>4.177419</x:v>
       </x:c>
       <x:c r="R21" s="3" t="n">
-        <x:v>4.579137</x:v>
+        <x:v>4.29661</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1931,52 +1931,52 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="C22" s="4" t="n">
-        <x:v>0.046120799999999997</x:v>
+        <x:v>0.03877428</x:v>
       </x:c>
       <x:c r="D22" s="4" t="n">
-        <x:v>-0.08276863000000001</x:v>
+        <x:v>-0.09114337</x:v>
       </x:c>
       <x:c r="E22" s="4" t="n">
-        <x:v>-0.024731640000000003</x:v>
+        <x:v>-0.025579960000000002</x:v>
       </x:c>
       <x:c r="F22" s="4" t="n">
-        <x:v>-0.14502652</x:v>
+        <x:v>-0.14765727</x:v>
       </x:c>
       <x:c r="G22" s="4" t="n">
-        <x:v>0.20191166</x:v>
+        <x:v>0.10108402</x:v>
       </x:c>
       <x:c r="H22" s="4" t="n">
-        <x:v>0.10237738</x:v>
+        <x:v>-0.00114726</x:v>
       </x:c>
       <x:c r="I22" s="4" t="n">
-        <x:v>-0.01199125</x:v>
+        <x:v>-0.020261909999999998</x:v>
       </x:c>
       <x:c r="J22" s="4" t="n">
-        <x:v>-0.10697424</x:v>
+        <x:v>-0.11959613</x:v>
       </x:c>
       <x:c r="K22" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L22" s="5" t="n">
-        <x:v>2825</x:v>
+        <x:v>3206</x:v>
       </x:c>
       <x:c r="M22" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N22" s="5" t="n">
-        <x:v>135</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="O22" s="3" t="n">
-        <x:v>4.38</x:v>
+        <x:v>4.300714</x:v>
       </x:c>
       <x:c r="P22" s="3" t="n">
-        <x:v>4.560088</x:v>
+        <x:v>4.432158</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="n">
-        <x:v>4.335526</x:v>
+        <x:v>4.341398</x:v>
       </x:c>
       <x:c r="R22" s="3" t="n">
-        <x:v>4.757407</x:v>
+        <x:v>4.465909</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1987,52 +1987,52 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="C23" s="4" t="n">
-        <x:v>0.04521025</x:v>
+        <x:v>0.03796687</x:v>
       </x:c>
       <x:c r="D23" s="4" t="n">
-        <x:v>-0.08444378000000001</x:v>
+        <x:v>-0.09190382</x:v>
       </x:c>
       <x:c r="E23" s="4" t="n">
-        <x:v>-0.023998330000000002</x:v>
+        <x:v>-0.0257983</x:v>
       </x:c>
       <x:c r="F23" s="4" t="n">
-        <x:v>-0.14541458000000002</x:v>
+        <x:v>-0.14839468</x:v>
       </x:c>
       <x:c r="G23" s="4" t="n">
-        <x:v>0.19800308</x:v>
+        <x:v>0.102569</x:v>
       </x:c>
       <x:c r="H23" s="4" t="n">
-        <x:v>0.09812398</x:v>
+        <x:v>-0.00209404</x:v>
       </x:c>
       <x:c r="I23" s="4" t="n">
-        <x:v>-0.01676229</x:v>
+        <x:v>-0.01739699</x:v>
       </x:c>
       <x:c r="J23" s="4" t="n">
-        <x:v>-0.11284015</x:v>
+        <x:v>-0.11426869999999999</x:v>
       </x:c>
       <x:c r="K23" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L23" s="5" t="n">
-        <x:v>2804</x:v>
+        <x:v>3208</x:v>
       </x:c>
       <x:c r="M23" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N23" s="5" t="n">
-        <x:v>137</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="O23" s="3" t="n">
-        <x:v>4.523704</x:v>
+        <x:v>4.438496</x:v>
       </x:c>
       <x:c r="P23" s="3" t="n">
-        <x:v>4.716209</x:v>
+        <x:v>4.584165</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="n">
-        <x:v>4.506579</x:v>
+        <x:v>4.502688</x:v>
       </x:c>
       <x:c r="R23" s="3" t="n">
-        <x:v>4.95438</x:v>
+        <x:v>4.653631</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2043,52 +2043,52 @@
         <x:v>5.75</x:v>
       </x:c>
       <x:c r="C24" s="4" t="n">
-        <x:v>0.04455558</x:v>
+        <x:v>0.03802991</x:v>
       </x:c>
       <x:c r="D24" s="4" t="n">
-        <x:v>-0.08521266000000001</x:v>
+        <x:v>-0.0918149</x:v>
       </x:c>
       <x:c r="E24" s="4" t="n">
-        <x:v>-0.02320891</x:v>
+        <x:v>-0.02377775</x:v>
       </x:c>
       <x:c r="F24" s="4" t="n">
-        <x:v>-0.14551841</x:v>
+        <x:v>-0.14685515999999998</x:v>
       </x:c>
       <x:c r="G24" s="4" t="n">
-        <x:v>0.19364667000000002</x:v>
+        <x:v>0.10212299</x:v>
       </x:c>
       <x:c r="H24" s="4" t="n">
-        <x:v>0.09152996</x:v>
+        <x:v>-0.0036168899999999998</x:v>
       </x:c>
       <x:c r="I24" s="4" t="n">
-        <x:v>-0.0090039</x:v>
+        <x:v>-0.03237457</x:v>
       </x:c>
       <x:c r="J24" s="4" t="n">
-        <x:v>-0.10432454999999999</x:v>
+        <x:v>-0.12993609</x:v>
       </x:c>
       <x:c r="K24" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L24" s="5" t="n">
-        <x:v>2778</x:v>
+        <x:v>3168</x:v>
       </x:c>
       <x:c r="M24" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N24" s="5" t="n">
-        <x:v>135</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="O24" s="3" t="n">
-        <x:v>4.661389</x:v>
+        <x:v>4.571132</x:v>
       </x:c>
       <x:c r="P24" s="3" t="n">
-        <x:v>4.862671</x:v>
+        <x:v>4.717961</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="n">
-        <x:v>4.671053</x:v>
+        <x:v>4.66129</x:v>
       </x:c>
       <x:c r="R24" s="3" t="n">
-        <x:v>5.135185</x:v>
+        <x:v>4.835635</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2099,52 +2099,52 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C25" s="4" t="n">
-        <x:v>0.04477558</x:v>
+        <x:v>0.03717769</x:v>
       </x:c>
       <x:c r="D25" s="4" t="n">
-        <x:v>-0.08517493999999999</x:v>
+        <x:v>-0.09270219</x:v>
       </x:c>
       <x:c r="E25" s="4" t="n">
-        <x:v>-0.02281281</x:v>
+        <x:v>-0.020898020000000003</x:v>
       </x:c>
       <x:c r="F25" s="4" t="n">
-        <x:v>-0.145875</x:v>
+        <x:v>-0.14474273999999998</x:v>
       </x:c>
       <x:c r="G25" s="4" t="n">
-        <x:v>0.1946548</x:v>
+        <x:v>0.10763365999999999</x:v>
       </x:c>
       <x:c r="H25" s="4" t="n">
-        <x:v>0.09248946999999999</x:v>
+        <x:v>0.00208508</x:v>
       </x:c>
       <x:c r="I25" s="4" t="n">
-        <x:v>-0.021601699999999998</x:v>
+        <x:v>-0.02959575</x:v>
       </x:c>
       <x:c r="J25" s="4" t="n">
-        <x:v>-0.11794807</x:v>
+        <x:v>-0.12804722999999998</x:v>
       </x:c>
       <x:c r="K25" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L25" s="5" t="n">
-        <x:v>2761</x:v>
+        <x:v>3137</x:v>
       </x:c>
       <x:c r="M25" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N25" s="5" t="n">
-        <x:v>137</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="O25" s="3" t="n">
-        <x:v>4.794444</x:v>
+        <x:v>4.700365</x:v>
       </x:c>
       <x:c r="P25" s="3" t="n">
-        <x:v>5.005704</x:v>
+        <x:v>4.846191</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="n">
-        <x:v>4.835526</x:v>
+        <x:v>4.819892</x:v>
       </x:c>
       <x:c r="R25" s="3" t="n">
-        <x:v>5.328467</x:v>
+        <x:v>4.988764</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2155,52 +2155,52 @@
         <x:v>6.25</x:v>
       </x:c>
       <x:c r="C26" s="4" t="n">
-        <x:v>0.04457363</x:v>
+        <x:v>0.03798813</x:v>
       </x:c>
       <x:c r="D26" s="4" t="n">
-        <x:v>-0.08581214</x:v>
+        <x:v>-0.091895</x:v>
       </x:c>
       <x:c r="E26" s="4" t="n">
-        <x:v>-0.020923709999999998</x:v>
+        <x:v>-0.01903801</x:v>
       </x:c>
       <x:c r="F26" s="4" t="n">
-        <x:v>-0.14449087</x:v>
+        <x:v>-0.14317090999999998</x:v>
       </x:c>
       <x:c r="G26" s="4" t="n">
-        <x:v>0.19301390000000002</x:v>
+        <x:v>0.10670315999999999</x:v>
       </x:c>
       <x:c r="H26" s="4" t="n">
-        <x:v>0.09077088</x:v>
+        <x:v>0.00201721</x:v>
       </x:c>
       <x:c r="I26" s="4" t="n">
-        <x:v>-0.01433485</x:v>
+        <x:v>-0.01865126</x:v>
       </x:c>
       <x:c r="J26" s="4" t="n">
-        <x:v>-0.11050867</x:v>
+        <x:v>-0.11717045000000001</x:v>
       </x:c>
       <x:c r="K26" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L26" s="5" t="n">
-        <x:v>2734</x:v>
+        <x:v>3111</x:v>
       </x:c>
       <x:c r="M26" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N26" s="5" t="n">
-        <x:v>132</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="O26" s="3" t="n">
-        <x:v>4.923611</x:v>
+        <x:v>4.824701</x:v>
       </x:c>
       <x:c r="P26" s="3" t="n">
-        <x:v>5.136247</x:v>
+        <x:v>4.96874</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="n">
-        <x:v>5</x:v>
+        <x:v>4.978495</x:v>
       </x:c>
       <x:c r="R26" s="3" t="n">
-        <x:v>5.479167</x:v>
+        <x:v>5.123563</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2211,52 +2211,52 @@
         <x:v>6.5</x:v>
       </x:c>
       <x:c r="C27" s="4" t="n">
-        <x:v>0.04501243</x:v>
+        <x:v>0.03817608</x:v>
       </x:c>
       <x:c r="D27" s="4" t="n">
-        <x:v>-0.08565292</x:v>
+        <x:v>-0.09218246000000001</x:v>
       </x:c>
       <x:c r="E27" s="4" t="n">
-        <x:v>-0.01922134</x:v>
+        <x:v>-0.02004941</x:v>
       </x:c>
       <x:c r="F27" s="4" t="n">
-        <x:v>-0.14310118</x:v>
+        <x:v>-0.14460314</x:v>
       </x:c>
       <x:c r="G27" s="4" t="n">
-        <x:v>0.19048948</x:v>
+        <x:v>0.10662413000000001</x:v>
       </x:c>
       <x:c r="H27" s="4" t="n">
-        <x:v>0.08589905999999999</x:v>
+        <x:v>-0.00021496000000000002</x:v>
       </x:c>
       <x:c r="I27" s="4" t="n">
-        <x:v>-0.021013860000000002</x:v>
+        <x:v>-0.0141459</x:v>
       </x:c>
       <x:c r="J27" s="4" t="n">
-        <x:v>-0.11914403999999999</x:v>
+        <x:v>-0.1147467</x:v>
       </x:c>
       <x:c r="K27" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L27" s="5" t="n">
-        <x:v>2706</x:v>
+        <x:v>3077</x:v>
       </x:c>
       <x:c r="M27" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N27" s="5" t="n">
-        <x:v>137</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="O27" s="3" t="n">
-        <x:v>5.046944</x:v>
+        <x:v>4.943144</x:v>
       </x:c>
       <x:c r="P27" s="3" t="n">
-        <x:v>5.259239</x:v>
+        <x:v>5.08141</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="n">
-        <x:v>5.161184</x:v>
+        <x:v>5.129032</x:v>
       </x:c>
       <x:c r="R27" s="3" t="n">
-        <x:v>5.677007</x:v>
+        <x:v>5.25</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2267,52 +2267,52 @@
         <x:v>6.75</x:v>
       </x:c>
       <x:c r="C28" s="4" t="n">
-        <x:v>0.04481364</x:v>
+        <x:v>0.03687593</x:v>
       </x:c>
       <x:c r="D28" s="4" t="n">
-        <x:v>-0.08625392</x:v>
+        <x:v>-0.09287456000000001</x:v>
       </x:c>
       <x:c r="E28" s="4" t="n">
-        <x:v>-0.01817877</x:v>
+        <x:v>-0.01833125</x:v>
       </x:c>
       <x:c r="F28" s="4" t="n">
-        <x:v>-0.14275758</x:v>
+        <x:v>-0.14265472</x:v>
       </x:c>
       <x:c r="G28" s="4" t="n">
-        <x:v>0.18689737</x:v>
+        <x:v>0.10173046</x:v>
       </x:c>
       <x:c r="H28" s="4" t="n">
-        <x:v>0.08106661000000001</x:v>
+        <x:v>-0.00541474</x:v>
       </x:c>
       <x:c r="I28" s="4" t="n">
-        <x:v>-0.01390664</x:v>
+        <x:v>-0.02595827</x:v>
       </x:c>
       <x:c r="J28" s="4" t="n">
-        <x:v>-0.11286602999999999</x:v>
+        <x:v>-0.12171636</x:v>
       </x:c>
       <x:c r="K28" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L28" s="5" t="n">
-        <x:v>2686</x:v>
+        <x:v>3072</x:v>
       </x:c>
       <x:c r="M28" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N28" s="5" t="n">
-        <x:v>131</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="O28" s="3" t="n">
-        <x:v>5.165093</x:v>
+        <x:v>5.056856</x:v>
       </x:c>
       <x:c r="P28" s="3" t="n">
-        <x:v>5.379561</x:v>
+        <x:v>5.200928</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="n">
-        <x:v>5.319079</x:v>
+        <x:v>5.274194</x:v>
       </x:c>
       <x:c r="R28" s="3" t="n">
-        <x:v>5.805344</x:v>
+        <x:v>5.447443</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2323,52 +2323,52 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C29" s="4" t="n">
-        <x:v>0.04393601999999999</x:v>
+        <x:v>0.03650442</x:v>
       </x:c>
       <x:c r="D29" s="4" t="n">
-        <x:v>-0.08724453</x:v>
+        <x:v>-0.09290055000000001</x:v>
       </x:c>
       <x:c r="E29" s="4" t="n">
-        <x:v>-0.018502559999999998</x:v>
+        <x:v>-0.01849069</x:v>
       </x:c>
       <x:c r="F29" s="4" t="n">
-        <x:v>-0.14385314</x:v>
+        <x:v>-0.14326427</x:v>
       </x:c>
       <x:c r="G29" s="4" t="n">
-        <x:v>0.1829887</x:v>
+        <x:v>0.09623461999999999</x:v>
       </x:c>
       <x:c r="H29" s="4" t="n">
-        <x:v>0.07626068</x:v>
+        <x:v>-0.00866334</x:v>
       </x:c>
       <x:c r="I29" s="4" t="n">
-        <x:v>-0.03023102</x:v>
+        <x:v>-0.02122512</x:v>
       </x:c>
       <x:c r="J29" s="4" t="n">
-        <x:v>-0.133162</x:v>
+        <x:v>-0.11650655</x:v>
       </x:c>
       <x:c r="K29" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L29" s="5" t="n">
-        <x:v>2663</x:v>
+        <x:v>3053</x:v>
       </x:c>
       <x:c r="M29" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N29" s="5" t="n">
-        <x:v>130</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="O29" s="3" t="n">
-        <x:v>5.279167</x:v>
+        <x:v>5.165671</x:v>
       </x:c>
       <x:c r="P29" s="3" t="n">
-        <x:v>5.491551</x:v>
+        <x:v>5.308303</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="n">
-        <x:v>5.473684</x:v>
+        <x:v>5.416667</x:v>
       </x:c>
       <x:c r="R29" s="3" t="n">
-        <x:v>5.961538</x:v>
+        <x:v>5.586207</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2379,52 +2379,52 @@
         <x:v>7.25</x:v>
       </x:c>
       <x:c r="C30" s="4" t="n">
-        <x:v>0.04432124</x:v>
+        <x:v>0.03703709</x:v>
       </x:c>
       <x:c r="D30" s="4" t="n">
-        <x:v>-0.08675118</x:v>
+        <x:v>-0.09310921</x:v>
       </x:c>
       <x:c r="E30" s="4" t="n">
-        <x:v>-0.01599435</x:v>
+        <x:v>-0.01978554</x:v>
       </x:c>
       <x:c r="F30" s="4" t="n">
-        <x:v>-0.14204597</x:v>
+        <x:v>-0.145908</x:v>
       </x:c>
       <x:c r="G30" s="4" t="n">
-        <x:v>0.17443730999999998</x:v>
+        <x:v>0.09322525000000001</x:v>
       </x:c>
       <x:c r="H30" s="4" t="n">
-        <x:v>0.07025065999999999</x:v>
+        <x:v>-0.01216923</x:v>
       </x:c>
       <x:c r="I30" s="4" t="n">
-        <x:v>-0.00695368</x:v>
+        <x:v>-0.01509431</x:v>
       </x:c>
       <x:c r="J30" s="4" t="n">
-        <x:v>-0.10940025</x:v>
+        <x:v>-0.11362365</x:v>
       </x:c>
       <x:c r="K30" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L30" s="5" t="n">
-        <x:v>2633</x:v>
+        <x:v>3039</x:v>
       </x:c>
       <x:c r="M30" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N30" s="5" t="n">
-        <x:v>124</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="O30" s="3" t="n">
-        <x:v>5.38713</x:v>
+        <x:v>5.270003</x:v>
       </x:c>
       <x:c r="P30" s="3" t="n">
-        <x:v>5.5921</x:v>
+        <x:v>5.412307</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="n">
-        <x:v>5.625</x:v>
+        <x:v>5.55914</x:v>
       </x:c>
       <x:c r="R30" s="3" t="n">
-        <x:v>6.064516</x:v>
+        <x:v>5.689349</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2435,52 +2435,52 @@
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="C31" s="4" t="n">
-        <x:v>0.04416962</x:v>
+        <x:v>0.03712462</x:v>
       </x:c>
       <x:c r="D31" s="4" t="n">
-        <x:v>-0.08724768</x:v>
+        <x:v>-0.09313074</x:v>
       </x:c>
       <x:c r="E31" s="4" t="n">
-        <x:v>-0.01603565</x:v>
+        <x:v>-0.01631262</x:v>
       </x:c>
       <x:c r="F31" s="4" t="n">
-        <x:v>-0.14238759</x:v>
+        <x:v>-0.14324496</x:v>
       </x:c>
       <x:c r="G31" s="4" t="n">
-        <x:v>0.17064354999999998</x:v>
+        <x:v>0.08946739000000001</x:v>
       </x:c>
       <x:c r="H31" s="4" t="n">
-        <x:v>0.06497098</x:v>
+        <x:v>-0.01480709</x:v>
       </x:c>
       <x:c r="I31" s="4" t="n">
-        <x:v>-0.017107090000000002</x:v>
+        <x:v>-0.011767240000000002</x:v>
       </x:c>
       <x:c r="J31" s="4" t="n">
-        <x:v>-0.11961812</x:v>
+        <x:v>-0.11593876</x:v>
       </x:c>
       <x:c r="K31" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L31" s="5" t="n">
-        <x:v>2619</x:v>
+        <x:v>3001</x:v>
       </x:c>
       <x:c r="M31" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N31" s="5" t="n">
-        <x:v>125</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="O31" s="3" t="n">
-        <x:v>5.491111</x:v>
+        <x:v>5.369273</x:v>
       </x:c>
       <x:c r="P31" s="3" t="n">
-        <x:v>5.694922</x:v>
+        <x:v>5.493835</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="n">
-        <x:v>5.776316</x:v>
+        <x:v>5.698925</x:v>
       </x:c>
       <x:c r="R31" s="3" t="n">
-        <x:v>6.226</x:v>
+        <x:v>5.818452</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2491,52 +2491,52 @@
         <x:v>7.75</x:v>
       </x:c>
       <x:c r="C32" s="4" t="n">
-        <x:v>0.04357692</x:v>
+        <x:v>0.037573180000000005</x:v>
       </x:c>
       <x:c r="D32" s="4" t="n">
-        <x:v>-0.08771672999999999</x:v>
+        <x:v>-0.09313634999999999</x:v>
       </x:c>
       <x:c r="E32" s="4" t="n">
-        <x:v>-0.01842446</x:v>
+        <x:v>-0.01744422</x:v>
       </x:c>
       <x:c r="F32" s="4" t="n">
-        <x:v>-0.14565065</x:v>
+        <x:v>-0.14448206</x:v>
       </x:c>
       <x:c r="G32" s="4" t="n">
-        <x:v>0.16984801000000002</x:v>
+        <x:v>0.08904442</x:v>
       </x:c>
       <x:c r="H32" s="4" t="n">
-        <x:v>0.06390123</x:v>
+        <x:v>-0.01611713</x:v>
       </x:c>
       <x:c r="I32" s="4" t="n">
-        <x:v>-0.01089751</x:v>
+        <x:v>-0.01223776</x:v>
       </x:c>
       <x:c r="J32" s="4" t="n">
-        <x:v>-0.11825642</x:v>
+        <x:v>-0.11680996</x:v>
       </x:c>
       <x:c r="K32" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L32" s="5" t="n">
-        <x:v>2621</x:v>
+        <x:v>2991</x:v>
       </x:c>
       <x:c r="M32" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N32" s="5" t="n">
-        <x:v>125</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="O32" s="3" t="n">
-        <x:v>5.589815</x:v>
+        <x:v>5.464309</x:v>
       </x:c>
       <x:c r="P32" s="3" t="n">
-        <x:v>5.804655</x:v>
+        <x:v>5.586677</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="n">
-        <x:v>5.924342</x:v>
+        <x:v>5.836022</x:v>
       </x:c>
       <x:c r="R32" s="3" t="n">
-        <x:v>6.376</x:v>
+        <x:v>5.949405</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2547,52 +2547,52 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="4" t="n">
-        <x:v>0.04451598</x:v>
+        <x:v>0.03854826</x:v>
       </x:c>
       <x:c r="D33" s="4" t="n">
-        <x:v>-0.08746663</x:v>
+        <x:v>-0.09283447</x:v>
       </x:c>
       <x:c r="E33" s="4" t="n">
-        <x:v>-0.01704149</x:v>
+        <x:v>-0.01864176</x:v>
       </x:c>
       <x:c r="F33" s="4" t="n">
-        <x:v>-0.14435053</x:v>
+        <x:v>-0.14585703</x:v>
       </x:c>
       <x:c r="G33" s="4" t="n">
-        <x:v>0.16951298999999997</x:v>
+        <x:v>0.09349705</x:v>
       </x:c>
       <x:c r="H33" s="4" t="n">
-        <x:v>0.062249679999999995</x:v>
+        <x:v>-0.013964840000000001</x:v>
       </x:c>
       <x:c r="I33" s="4" t="n">
-        <x:v>-0.01311986</x:v>
+        <x:v>-0.02496233</x:v>
       </x:c>
       <x:c r="J33" s="4" t="n">
-        <x:v>-0.12116211</x:v>
+        <x:v>-0.12988058</x:v>
       </x:c>
       <x:c r="K33" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L33" s="5" t="n">
-        <x:v>2596</x:v>
+        <x:v>2989</x:v>
       </x:c>
       <x:c r="M33" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N33" s="5" t="n">
-        <x:v>124</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="O33" s="3" t="n">
-        <x:v>5.685185</x:v>
+        <x:v>5.556192</x:v>
       </x:c>
       <x:c r="P33" s="3" t="n">
-        <x:v>5.887712</x:v>
+        <x:v>5.681415</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="n">
-        <x:v>6.069079</x:v>
+        <x:v>5.973118</x:v>
       </x:c>
       <x:c r="R33" s="3" t="n">
-        <x:v>6.504032</x:v>
+        <x:v>6.134393</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2603,52 +2603,52 @@
         <x:v>8.25</x:v>
       </x:c>
       <x:c r="C34" s="4" t="n">
-        <x:v>0.044878270000000005</x:v>
+        <x:v>0.03833011</x:v>
       </x:c>
       <x:c r="D34" s="4" t="n">
-        <x:v>-0.08753875000000001</x:v>
+        <x:v>-0.09293456000000001</x:v>
       </x:c>
       <x:c r="E34" s="4" t="n">
-        <x:v>-0.0137131</x:v>
+        <x:v>-0.01630135</x:v>
       </x:c>
       <x:c r="F34" s="4" t="n">
-        <x:v>-0.14165192</x:v>
+        <x:v>-0.1440824</x:v>
       </x:c>
       <x:c r="G34" s="4" t="n">
-        <x:v>0.16451618</x:v>
+        <x:v>0.08899962</x:v>
       </x:c>
       <x:c r="H34" s="4" t="n">
-        <x:v>0.05706486</x:v>
+        <x:v>-0.01855711</x:v>
       </x:c>
       <x:c r="I34" s="4" t="n">
-        <x:v>-0.0067766300000000005</x:v>
+        <x:v>-0.01136801</x:v>
       </x:c>
       <x:c r="J34" s="4" t="n">
-        <x:v>-0.11531568</x:v>
+        <x:v>-0.11655707</x:v>
       </x:c>
       <x:c r="K34" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L34" s="5" t="n">
-        <x:v>2569</x:v>
+        <x:v>2963</x:v>
       </x:c>
       <x:c r="M34" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N34" s="5" t="n">
-        <x:v>123</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="O34" s="3" t="n">
-        <x:v>5.77713</x:v>
+        <x:v>5.645169</x:v>
       </x:c>
       <x:c r="P34" s="3" t="n">
-        <x:v>5.962923</x:v>
+        <x:v>5.753206</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="n">
-        <x:v>6.213816</x:v>
+        <x:v>6.110215</x:v>
       </x:c>
       <x:c r="R34" s="3" t="n">
-        <x:v>6.628049</x:v>
+        <x:v>6.229412</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2659,52 +2659,52 @@
         <x:v>8.5</x:v>
       </x:c>
       <x:c r="C35" s="4" t="n">
-        <x:v>0.04458181</x:v>
+        <x:v>0.03871019</x:v>
       </x:c>
       <x:c r="D35" s="4" t="n">
-        <x:v>-0.08779089000000001</x:v>
+        <x:v>-0.09300685</x:v>
       </x:c>
       <x:c r="E35" s="4" t="n">
-        <x:v>-0.01362201</x:v>
+        <x:v>-0.01614221</x:v>
       </x:c>
       <x:c r="F35" s="4" t="n">
-        <x:v>-0.14188335</x:v>
+        <x:v>-0.14433813</x:v>
       </x:c>
       <x:c r="G35" s="4" t="n">
-        <x:v>0.16036407</x:v>
+        <x:v>0.08629096</x:v>
       </x:c>
       <x:c r="H35" s="4" t="n">
-        <x:v>0.05149625</x:v>
+        <x:v>-0.02297731</x:v>
       </x:c>
       <x:c r="I35" s="4" t="n">
-        <x:v>-0.00553342</x:v>
+        <x:v>-0.01323941</x:v>
       </x:c>
       <x:c r="J35" s="4" t="n">
-        <x:v>-0.11499204</x:v>
+        <x:v>-0.1214541</x:v>
       </x:c>
       <x:c r="K35" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L35" s="5" t="n">
-        <x:v>2572</x:v>
+        <x:v>2962</x:v>
       </x:c>
       <x:c r="M35" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N35" s="5" t="n">
-        <x:v>122</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="O35" s="3" t="n">
-        <x:v>5.86537</x:v>
+        <x:v>5.730163</x:v>
       </x:c>
       <x:c r="P35" s="3" t="n">
-        <x:v>6.059778</x:v>
+        <x:v>5.840817</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="n">
-        <x:v>6.358553</x:v>
+        <x:v>6.247312</x:v>
       </x:c>
       <x:c r="R35" s="3" t="n">
-        <x:v>6.745902</x:v>
+        <x:v>6.301205</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2715,52 +2715,52 @@
         <x:v>8.75</x:v>
       </x:c>
       <x:c r="C36" s="4" t="n">
-        <x:v>0.04500741</x:v>
+        <x:v>0.03928761</x:v>
       </x:c>
       <x:c r="D36" s="4" t="n">
-        <x:v>-0.08771841</x:v>
+        <x:v>-0.09262549999999999</x:v>
       </x:c>
       <x:c r="E36" s="4" t="n">
-        <x:v>-0.01394491</x:v>
+        <x:v>-0.01631472</x:v>
       </x:c>
       <x:c r="F36" s="4" t="n">
-        <x:v>-0.1425958</x:v>
+        <x:v>-0.14515166000000002</x:v>
       </x:c>
       <x:c r="G36" s="4" t="n">
-        <x:v>0.15462504</x:v>
+        <x:v>0.08590829</x:v>
       </x:c>
       <x:c r="H36" s="4" t="n">
-        <x:v>0.04532014</x:v>
+        <x:v>-0.022638630000000003</x:v>
       </x:c>
       <x:c r="I36" s="4" t="n">
-        <x:v>-0.0051633600000000005</x:v>
+        <x:v>-0.00594807</x:v>
       </x:c>
       <x:c r="J36" s="4" t="n">
-        <x:v>-0.11513861</x:v>
+        <x:v>-0.11605771000000001</x:v>
       </x:c>
       <x:c r="K36" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L36" s="5" t="n">
-        <x:v>2562</x:v>
+        <x:v>2955</x:v>
       </x:c>
       <x:c r="M36" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N36" s="5" t="n">
-        <x:v>120</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="O36" s="3" t="n">
-        <x:v>5.95</x:v>
+        <x:v>5.812334</x:v>
       </x:c>
       <x:c r="P36" s="3" t="n">
-        <x:v>6.140515</x:v>
+        <x:v>5.919459</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="n">
-        <x:v>6.5</x:v>
+        <x:v>6.379032</x:v>
       </x:c>
       <x:c r="R36" s="3" t="n">
-        <x:v>6.839583</x:v>
+        <x:v>6.38872</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2771,52 +2771,52 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="4" t="n">
-        <x:v>0.04549443</x:v>
+        <x:v>0.03955422</x:v>
       </x:c>
       <x:c r="D37" s="4" t="n">
-        <x:v>-0.08754873999999999</x:v>
+        <x:v>-0.09267547000000001</x:v>
       </x:c>
       <x:c r="E37" s="4" t="n">
-        <x:v>-0.013980999999999999</x:v>
+        <x:v>-0.01610536</x:v>
       </x:c>
       <x:c r="F37" s="4" t="n">
-        <x:v>-0.14325912000000002</x:v>
+        <x:v>-0.14512629999999999</x:v>
       </x:c>
       <x:c r="G37" s="4" t="n">
-        <x:v>0.15185879</x:v>
+        <x:v>0.08521068</x:v>
       </x:c>
       <x:c r="H37" s="4" t="n">
-        <x:v>0.04225671</x:v>
+        <x:v>-0.024035630000000002</x:v>
       </x:c>
       <x:c r="I37" s="4" t="n">
-        <x:v>0.00406439</x:v>
+        <x:v>0.00073986</x:v>
       </x:c>
       <x:c r="J37" s="4" t="n">
-        <x:v>-0.10706028999999999</x:v>
+        <x:v>-0.11025055</x:v>
       </x:c>
       <x:c r="K37" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L37" s="5" t="n">
-        <x:v>2555</x:v>
+        <x:v>2952</x:v>
       </x:c>
       <x:c r="M37" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N37" s="5" t="n">
-        <x:v>117</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="O37" s="3" t="n">
-        <x:v>6.031759</x:v>
+        <x:v>5.890438</x:v>
       </x:c>
       <x:c r="P37" s="3" t="n">
-        <x:v>6.21908</x:v>
+        <x:v>5.997798</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="n">
-        <x:v>6.631579</x:v>
+        <x:v>6.505376</x:v>
       </x:c>
       <x:c r="R37" s="3" t="n">
-        <x:v>6.903846</x:v>
+        <x:v>6.4375</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2827,52 +2827,52 @@
         <x:v>9.25</x:v>
       </x:c>
       <x:c r="C38" s="4" t="n">
-        <x:v>0.045434970000000005</x:v>
+        <x:v>0.03998207</x:v>
       </x:c>
       <x:c r="D38" s="4" t="n">
-        <x:v>-0.08764687</x:v>
+        <x:v>-0.09224942</x:v>
       </x:c>
       <x:c r="E38" s="4" t="n">
-        <x:v>-0.01348161</x:v>
+        <x:v>-0.01381031</x:v>
       </x:c>
       <x:c r="F38" s="4" t="n">
-        <x:v>-0.14300353</x:v>
+        <x:v>-0.14342328000000001</x:v>
       </x:c>
       <x:c r="G38" s="4" t="n">
-        <x:v>0.14795714000000001</x:v>
+        <x:v>0.08404049000000001</x:v>
       </x:c>
       <x:c r="H38" s="4" t="n">
-        <x:v>0.03792561</x:v>
+        <x:v>-0.026391170000000002</x:v>
       </x:c>
       <x:c r="I38" s="4" t="n">
-        <x:v>-0.00267833</x:v>
+        <x:v>-0.00571465</x:v>
       </x:c>
       <x:c r="J38" s="4" t="n">
-        <x:v>-0.11350634</x:v>
+        <x:v>-0.11653191</x:v>
       </x:c>
       <x:c r="K38" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L38" s="5" t="n">
-        <x:v>2548</x:v>
+        <x:v>2921</x:v>
       </x:c>
       <x:c r="M38" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N38" s="5" t="n">
-        <x:v>119</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="O38" s="3" t="n">
-        <x:v>6.11</x:v>
+        <x:v>5.965388</x:v>
       </x:c>
       <x:c r="P38" s="3" t="n">
-        <x:v>6.293171</x:v>
+        <x:v>6.042537</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="n">
-        <x:v>6.763158</x:v>
+        <x:v>6.63172</x:v>
       </x:c>
       <x:c r="R38" s="3" t="n">
-        <x:v>7.054622</x:v>
+        <x:v>6.562112</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2883,52 +2883,52 @@
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="C39" s="4" t="n">
-        <x:v>0.04574687</x:v>
+        <x:v>0.03963278</x:v>
       </x:c>
       <x:c r="D39" s="4" t="n">
-        <x:v>-0.08725006</x:v>
+        <x:v>-0.09205619000000001</x:v>
       </x:c>
       <x:c r="E39" s="4" t="n">
-        <x:v>-0.01206821</x:v>
+        <x:v>-0.014260219999999999</x:v>
       </x:c>
       <x:c r="F39" s="4" t="n">
-        <x:v>-0.14225091</x:v>
+        <x:v>-0.14394686</x:v>
       </x:c>
       <x:c r="G39" s="4" t="n">
-        <x:v>0.14639452</x:v>
+        <x:v>0.08521092</x:v>
       </x:c>
       <x:c r="H39" s="4" t="n">
-        <x:v>0.0357702</x:v>
+        <x:v>-0.02499568</x:v>
       </x:c>
       <x:c r="I39" s="4" t="n">
-        <x:v>-0.00307268</x:v>
+        <x:v>-0.012642</x:v>
       </x:c>
       <x:c r="J39" s="4" t="n">
-        <x:v>-0.11531788000000001</x:v>
+        <x:v>-0.12143888</x:v>
       </x:c>
       <x:c r="K39" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L39" s="5" t="n">
-        <x:v>2530</x:v>
+        <x:v>2920</x:v>
       </x:c>
       <x:c r="M39" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N39" s="5" t="n">
-        <x:v>118</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="O39" s="3" t="n">
-        <x:v>6.185185</x:v>
+        <x:v>6.038264</x:v>
       </x:c>
       <x:c r="P39" s="3" t="n">
-        <x:v>6.349209</x:v>
+        <x:v>6.114983</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="n">
-        <x:v>6.894737</x:v>
+        <x:v>6.758065</x:v>
       </x:c>
       <x:c r="R39" s="3" t="n">
-        <x:v>7.148305</x:v>
+        <x:v>6.70092</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2939,52 +2939,52 @@
         <x:v>9.75</x:v>
       </x:c>
       <x:c r="C40" s="4" t="n">
-        <x:v>0.04586551</x:v>
+        <x:v>0.04009554</x:v>
       </x:c>
       <x:c r="D40" s="4" t="n">
-        <x:v>-0.08703288</x:v>
+        <x:v>-0.09202363999999999</x:v>
       </x:c>
       <x:c r="E40" s="4" t="n">
-        <x:v>-0.0129453</x:v>
+        <x:v>-0.01381454</x:v>
       </x:c>
       <x:c r="F40" s="4" t="n">
-        <x:v>-0.14332185</x:v>
+        <x:v>-0.14406373</x:v>
       </x:c>
       <x:c r="G40" s="4" t="n">
-        <x:v>0.14473527</x:v>
+        <x:v>0.08327712</x:v>
       </x:c>
       <x:c r="H40" s="4" t="n">
-        <x:v>0.034069630000000004</x:v>
+        <x:v>-0.02722147</x:v>
       </x:c>
       <x:c r="I40" s="4" t="n">
-        <x:v>-0.0022140199999999997</x:v>
+        <x:v>-0.00840409</x:v>
       </x:c>
       <x:c r="J40" s="4" t="n">
-        <x:v>-0.11525044</x:v>
+        <x:v>-0.11840706000000001</x:v>
       </x:c>
       <x:c r="K40" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L40" s="5" t="n">
-        <x:v>2534</x:v>
+        <x:v>2917</x:v>
       </x:c>
       <x:c r="M40" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N40" s="5" t="n">
-        <x:v>116</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="O40" s="3" t="n">
-        <x:v>6.257963</x:v>
+        <x:v>6.107736</x:v>
       </x:c>
       <x:c r="P40" s="3" t="n">
-        <x:v>6.428473</x:v>
+        <x:v>6.182036</x:v>
       </x:c>
       <x:c r="Q40" s="3" t="n">
-        <x:v>7.026316</x:v>
+        <x:v>6.88172</x:v>
       </x:c>
       <x:c r="R40" s="3" t="n">
-        <x:v>7.213362</x:v>
+        <x:v>6.75</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2995,59 +2995,59 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C41" s="4" t="n">
-        <x:v>0.04615957</x:v>
+        <x:v>0.04028342</x:v>
       </x:c>
       <x:c r="D41" s="4" t="n">
-        <x:v>-0.08705237</x:v>
+        <x:v>-0.09222559999999999</x:v>
       </x:c>
       <x:c r="E41" s="4" t="n">
-        <x:v>-0.01325015</x:v>
+        <x:v>-0.01471164</x:v>
       </x:c>
       <x:c r="F41" s="4" t="n">
-        <x:v>-0.14394679</x:v>
+        <x:v>-0.14535553</x:v>
       </x:c>
       <x:c r="G41" s="4" t="n">
-        <x:v>0.1437518</x:v>
+        <x:v>0.08579261</x:v>
       </x:c>
       <x:c r="H41" s="4" t="n">
-        <x:v>0.03233765</x:v>
+        <x:v>-0.025919650000000002</x:v>
       </x:c>
       <x:c r="I41" s="4" t="n">
-        <x:v>0.00519944</x:v>
+        <x:v>-0.00772301</x:v>
       </x:c>
       <x:c r="J41" s="4" t="n">
-        <x:v>-0.10899497999999999</x:v>
+        <x:v>-0.11951645</x:v>
       </x:c>
       <x:c r="K41" s="5" t="n">
-        <x:v>2700</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="L41" s="5" t="n">
-        <x:v>2541</x:v>
+        <x:v>2919</x:v>
       </x:c>
       <x:c r="M41" s="5" t="n">
-        <x:v>76</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="N41" s="5" t="n">
-        <x:v>114</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="O41" s="3" t="n">
-        <x:v>6.327315</x:v>
+        <x:v>6.175299</x:v>
       </x:c>
       <x:c r="P41" s="3" t="n">
-        <x:v>6.509445</x:v>
+        <x:v>6.251456</x:v>
       </x:c>
       <x:c r="Q41" s="3" t="n">
-        <x:v>7.154605</x:v>
+        <x:v>7.005376</x:v>
       </x:c>
       <x:c r="R41" s="3" t="n">
-        <x:v>7.27193</x:v>
+        <x:v>6.808544</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d0d43b70f554158"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6c401c50ad74cc4"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d53d35483024bf5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6321ca53d17c4ba8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>